<commit_message>
fix: complete optimization scope repair and paper evidence
</commit_message>
<xml_diff>
--- a/training/2021_C_round2_retry1/outputs/附件A 订购方案数据结果.xlsx
+++ b/training/2021_C_round2_retry1/outputs/附件A 订购方案数据结果.xlsx
@@ -2948,76 +2948,76 @@
         <v>65</v>
       </c>
       <c r="B43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="C43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="K43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="L43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="M43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="N43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="O43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="P43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="Q43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="R43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="S43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="T43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="U43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="V43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="W43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="X43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
       <c r="Y43" s="6" t="n">
-        <v>420.354037267081</v>
+        <v>420.35403726708</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5055,76 +5055,76 @@
         <v>136</v>
       </c>
       <c r="B114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="C114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="F114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="G114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="H114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="I114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="J114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="K114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="L114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="M114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="N114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="O114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="P114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="Q114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="R114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="S114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="T114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="U114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="V114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="W114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="X114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
       <c r="Y114" s="6" t="n">
-        <v>1131.02083333333</v>
+        <v>1084.60601072492</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5818,76 +5818,76 @@
         <v>159</v>
       </c>
       <c r="B137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="C137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="D137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="E137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="F137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="G137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="H137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="I137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="J137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="K137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="L137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="M137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="N137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="O137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="P137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="Q137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="R137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="S137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="T137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="U137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="V137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="W137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="X137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
       <c r="Y137" s="6" t="n">
-        <v>580.554394780335</v>
+        <v>580.554394798827</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7885,76 +7885,76 @@
         <v>222</v>
       </c>
       <c r="B200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="C200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="D200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="E200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="F200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="G200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="H200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="I200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="J200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="K200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="L200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="M200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="N200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="O200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="P200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="Q200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="R200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="S200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="T200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="U200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="V200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="W200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="X200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
       <c r="Y200" s="6" t="n">
-        <v>422.41653202927</v>
+        <v>422.41653198679</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10474,76 +10474,76 @@
         <v>303</v>
       </c>
       <c r="B281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="C281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="D281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="E281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="F281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="G281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="H281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="I281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="J281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="K281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="L281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="M281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="N281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="O281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="P281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="Q281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="R281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="S281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="T281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="U281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="V281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="W281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="X281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
       <c r="Y281" s="6" t="n">
-        <v>655.148868909483</v>
+        <v>660.637500002564</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11546,76 +11546,76 @@
         <v>335</v>
       </c>
       <c r="B313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="C313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="D313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="E313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="F313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="G313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="H313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="I313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="J313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="K313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="L313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="M313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="N313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="O313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="P313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="Q313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="R313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="S313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="T313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="U313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="V313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="W313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="X313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
       <c r="Y313" s="6" t="n">
-        <v>592.924418604661</v>
+        <v>585.766161633266</v>
       </c>
     </row>
     <row r="314" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12357,76 +12357,76 @@
         <v>358</v>
       </c>
       <c r="B336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="C336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="D336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="E336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="F336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="G336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="H336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="I336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="J336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="K336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="L336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="M336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="N336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="O336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="P336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="Q336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="R336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="S336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="T336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="U336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="V336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="W336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="X336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
       <c r="Y336" s="6" t="n">
-        <v>720.749999999982</v>
+        <v>720.75</v>
       </c>
     </row>
     <row r="337" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12695,76 +12695,76 @@
         <v>368</v>
       </c>
       <c r="B346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="C346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="D346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="E346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="F346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="G346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="H346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="I346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="J346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="K346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="L346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="M346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="N346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="O346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="P346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="Q346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="R346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="S346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="T346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="U346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="V346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="W346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="X346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
       <c r="Y346" s="6" t="n">
-        <v>675.328278914105</v>
+        <v>716.666666666667</v>
       </c>
     </row>
     <row r="347" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12975,76 +12975,76 @@
         <v>376</v>
       </c>
       <c r="B354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="C354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="D354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="E354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="F354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="G354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="H354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="I354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="J354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="K354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="L354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="M354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="N354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="O354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="P354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="Q354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="R354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="S354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="T354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="U354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="V354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="W354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="X354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
       <c r="Y354" s="6" t="n">
-        <v>839.743718592965</v>
+        <v>839.743718587589</v>
       </c>
     </row>
     <row r="355" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14811,99 +14811,99 @@
       </c>
       <c r="B409" s="3" t="n">
         <f aca="false">SUM(B7:B408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="C409" s="2" t="n">
         <f aca="false">SUM(C7:C408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="D409" s="3" t="n">
         <f aca="false">SUM(D7:D408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="E409" s="2" t="n">
         <f aca="false">SUM(E7:E408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="F409" s="3" t="n">
         <f aca="false">SUM(F7:F408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="G409" s="2" t="n">
         <f aca="false">SUM(G7:G408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="H409" s="3" t="n">
         <f aca="false">SUM(H7:H408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="I409" s="2" t="n">
         <f aca="false">SUM(I7:I408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="J409" s="3" t="n">
         <f aca="false">SUM(J7:J408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="K409" s="2" t="n">
         <f aca="false">SUM(K7:K408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="L409" s="3" t="n">
         <f aca="false">SUM(L7:L408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="M409" s="2" t="n">
         <f aca="false">SUM(M7:M408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="N409" s="3" t="n">
         <f aca="false">SUM(N7:N408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="O409" s="2" t="n">
         <f aca="false">SUM(O7:O408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="P409" s="3" t="n">
         <f aca="false">SUM(P7:P408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="Q409" s="2" t="n">
         <f aca="false">SUM(Q7:Q408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="R409" s="3" t="n">
         <f aca="false">SUM(R7:R408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="S409" s="2" t="n">
         <f aca="false">SUM(S7:S408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="T409" s="3" t="n">
         <f aca="false">SUM(T7:T408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="U409" s="2" t="n">
         <f aca="false">SUM(U7:U408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="V409" s="3" t="n">
         <f aca="false">SUM(V7:V408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="W409" s="2" t="n">
         <f aca="false">SUM(W7:W408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="X409" s="3" t="n">
         <f aca="false">SUM(X7:X408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
       <c r="Y409" s="2" t="n">
         <f aca="false">SUM(Y7:Y408)</f>
-        <v>27467.291523062</v>
+        <v>27460.5454622985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>